<commit_message>
Consult. libérales : import date consultation + date bloc (sans médecin)
Le fichier ne contient pas de colonne médecin : chaque ligne relie une
date de consultation à une date de bloc opératoire. Le MAR de la
consultation libérale du jour opère le patient :
- il doit être disponible à la date de bloc (sinon écarté du créneau) ;
- il est au bloc ce jour-là, donc sans consultation (même semaine
  comprise).
Remplace la notion de présence requise par médecin ; tableau de
contrôle par patient, marqueur 🩺 dans le planning, modèle Excel mis à
jour.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QYquHqHnHVYDevi2KPcbaN
</commit_message>
<xml_diff>
--- a/modele_consultations_liberales.xlsx
+++ b/modele_consultations_liberales.xlsx
@@ -400,17 +400,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C4"/>
   <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
     <col min="3" max="3" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Date</v>
+        <v>Date consultation</v>
       </c>
       <c r="B1" t="str">
-        <v>Médecin</v>
+        <v>Date bloc opératoire</v>
       </c>
       <c r="C1" t="str">
         <v>Examen</v>
@@ -420,8 +420,8 @@
       <c r="A2" s="1">
         <v>46308</v>
       </c>
-      <c r="B2" t="str">
-        <v>RW</v>
+      <c r="B2" s="1">
+        <v>46314</v>
       </c>
       <c r="C2" t="str">
         <v>Coloscopie</v>
@@ -431,8 +431,8 @@
       <c r="A3" s="1">
         <v>46317</v>
       </c>
-      <c r="B3" t="str">
-        <v>SG</v>
+      <c r="B3" s="1">
+        <v>46322</v>
       </c>
       <c r="C3" t="str">
         <v>Gastroscopie</v>
@@ -442,8 +442,8 @@
       <c r="A4" s="1">
         <v>46350</v>
       </c>
-      <c r="B4" t="str">
-        <v>GR</v>
+      <c r="B4" s="1">
+        <v>46356</v>
       </c>
       <c r="C4" t="str">
         <v>Écho-endoscopie</v>

</xml_diff>